<commit_message>
new driver data added
</commit_message>
<xml_diff>
--- a/public/media/import/driver_data.xlsx
+++ b/public/media/import/driver_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Admin360\Vehicle\Data to import\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\admin360\public\media\import\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A5D10B3F-7E60-40F6-B579-D9BF270D78D0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B258613-35C7-42FF-9515-44B348F3F8A5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9684" xr2:uid="{36D14F7D-3ED8-4450-9A04-4492755BE6E4}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{0E7C3F4B-CC9D-4B2C-9A31-05B8B024AA97}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1636,7 +1636,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEDD0202-C8DA-4A6C-8F16-5C29E6F609CF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8E4EC86-453F-49BD-8D81-FFFFFD3DDC72}">
   <dimension ref="A1:AC185"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>